<commit_message>
062425 - updating skins
</commit_message>
<xml_diff>
--- a/public/results/2025/Week 5 Skins.xlsx
+++ b/public/results/2025/Week 5 Skins.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amentumcms-my.sharepoint.com/personal/mark_hutter_amentumcms_com/Documents/DATA/Code/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="8_{0B9D84DB-407C-4044-A017-7F1E80D6798E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4F8F6CA4-3589-4BE2-81BE-C2CE95A69AEC}"/>
+  <xr:revisionPtr revIDLastSave="44" documentId="8_{0B9D84DB-407C-4044-A017-7F1E80D6798E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{275558B3-E703-4730-B3AA-E2C2851A63C9}"/>
   <bookViews>
-    <workbookView xWindow="7965" yWindow="1365" windowWidth="26730" windowHeight="18000" xr2:uid="{FDD4B5AF-41DC-445C-958F-C2DE65610468}"/>
+    <workbookView xWindow="7950" yWindow="2865" windowWidth="26730" windowHeight="18000" xr2:uid="{FDD4B5AF-41DC-445C-958F-C2DE65610468}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 5 Skins" sheetId="1" r:id="rId1"/>
@@ -53,9 +53,6 @@
     <t>Hole</t>
   </si>
   <si>
-    <t>Hdcp</t>
-  </si>
-  <si>
     <t>PAR</t>
   </si>
   <si>
@@ -98,16 +95,19 @@
     <t>Ige (.5)</t>
   </si>
   <si>
-    <t>Ige, Shayne (21)</t>
-  </si>
-  <si>
-    <t>Walters, Kevin (17)</t>
-  </si>
-  <si>
-    <t>Bess, John (15)</t>
-  </si>
-  <si>
-    <t>Young, Mark (13)</t>
+    <t>Mark Y</t>
+  </si>
+  <si>
+    <t>John B</t>
+  </si>
+  <si>
+    <t>Kevin W</t>
+  </si>
+  <si>
+    <t>Shayne I</t>
+  </si>
+  <si>
+    <t>HDCP</t>
   </si>
 </sst>
 </file>
@@ -118,7 +118,7 @@
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -165,6 +165,25 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -198,7 +217,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -341,19 +360,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFAEABAB"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FFAEABAB"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFAEABAB"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -474,6 +480,43 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFAEABAB"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFAEABAB"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFAEABAB"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -484,14 +527,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -501,13 +538,7 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -516,32 +547,17 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -549,66 +565,109 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="8" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="8" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -627,6 +686,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -949,763 +1012,766 @@
   <dimension ref="A1:O19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" customWidth="1"/>
-    <col min="3" max="11" width="10.7109375" customWidth="1"/>
-    <col min="12" max="12" width="6.7109375" customWidth="1"/>
-    <col min="13" max="13" width="5.7109375" style="43" customWidth="1"/>
-    <col min="14" max="14" width="7.5703125" style="43" customWidth="1"/>
-    <col min="15" max="15" width="8.140625" style="43" customWidth="1"/>
+    <col min="1" max="1" width="10.28515625" style="28" customWidth="1"/>
+    <col min="2" max="2" width="9.5703125" style="28" customWidth="1"/>
+    <col min="3" max="11" width="8.7109375" style="28" customWidth="1"/>
+    <col min="12" max="12" width="4" style="28" customWidth="1"/>
+    <col min="13" max="13" width="5.7109375" style="28" customWidth="1"/>
+    <col min="14" max="14" width="7" style="28" customWidth="1"/>
+    <col min="15" max="15" width="6.7109375" style="28" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-      <c r="M1" s="3" t="s">
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="38"/>
+      <c r="H1" s="38"/>
+      <c r="I1" s="38"/>
+      <c r="J1" s="38"/>
+      <c r="K1" s="38"/>
+      <c r="L1" s="38"/>
+      <c r="M1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="N1" s="4"/>
-      <c r="O1" s="5" t="s">
+      <c r="N1" s="2"/>
+      <c r="O1" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="7">
+      <c r="B2" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="4">
         <v>1</v>
       </c>
-      <c r="D2" s="7">
-        <v>2</v>
-      </c>
-      <c r="E2" s="7">
+      <c r="D2" s="4">
+        <v>2</v>
+      </c>
+      <c r="E2" s="4">
         <v>3</v>
       </c>
-      <c r="F2" s="7">
-        <v>4</v>
-      </c>
-      <c r="G2" s="7">
+      <c r="F2" s="4">
+        <v>4</v>
+      </c>
+      <c r="G2" s="4">
         <v>5</v>
       </c>
-      <c r="H2" s="7">
-        <v>6</v>
-      </c>
-      <c r="I2" s="7">
+      <c r="H2" s="4">
+        <v>6</v>
+      </c>
+      <c r="I2" s="4">
         <v>7</v>
       </c>
-      <c r="J2" s="7">
+      <c r="J2" s="4">
         <v>8</v>
       </c>
-      <c r="K2" s="7">
+      <c r="K2" s="4">
         <v>9</v>
       </c>
-      <c r="L2" s="8" t="s">
+      <c r="L2" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="M2" s="5"/>
+      <c r="N2" s="6"/>
+      <c r="O2" s="24"/>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" s="40"/>
+      <c r="B3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="M2" s="9"/>
-      <c r="N2" s="10"/>
-      <c r="O2" s="39"/>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="11"/>
-      <c r="B3" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="12">
-        <v>4</v>
-      </c>
-      <c r="D3" s="12">
+      <c r="C3" s="7">
+        <v>4</v>
+      </c>
+      <c r="D3" s="7">
         <v>5</v>
       </c>
-      <c r="E3" s="12">
-        <v>4</v>
-      </c>
-      <c r="F3" s="12">
+      <c r="E3" s="7">
+        <v>4</v>
+      </c>
+      <c r="F3" s="7">
         <v>3</v>
       </c>
-      <c r="G3" s="12">
-        <v>4</v>
-      </c>
-      <c r="H3" s="12">
-        <v>4</v>
-      </c>
-      <c r="I3" s="12">
+      <c r="G3" s="7">
+        <v>4</v>
+      </c>
+      <c r="H3" s="7">
+        <v>4</v>
+      </c>
+      <c r="I3" s="7">
         <v>3</v>
       </c>
-      <c r="J3" s="12">
-        <v>4</v>
-      </c>
-      <c r="K3" s="12">
+      <c r="J3" s="7">
+        <v>4</v>
+      </c>
+      <c r="K3" s="7">
         <v>5</v>
       </c>
-      <c r="L3" s="13"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="15"/>
-      <c r="O3" s="40"/>
+      <c r="L3" s="31"/>
+      <c r="M3" s="8"/>
+      <c r="N3" s="9"/>
+      <c r="O3" s="25"/>
     </row>
     <row r="4" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="16"/>
-      <c r="B4" s="17" t="s">
+      <c r="A4" s="41"/>
+      <c r="B4" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="10">
+        <v>4</v>
+      </c>
+      <c r="D4" s="10">
+        <v>1</v>
+      </c>
+      <c r="E4" s="10">
+        <v>3</v>
+      </c>
+      <c r="F4" s="10">
+        <v>9</v>
+      </c>
+      <c r="G4" s="10">
+        <v>5</v>
+      </c>
+      <c r="H4" s="10">
         <v>7</v>
       </c>
-      <c r="C4" s="17">
-        <v>4</v>
-      </c>
-      <c r="D4" s="17">
-        <v>1</v>
-      </c>
-      <c r="E4" s="17">
+      <c r="I4" s="10">
+        <v>8</v>
+      </c>
+      <c r="J4" s="10">
+        <v>6</v>
+      </c>
+      <c r="K4" s="10">
+        <v>2</v>
+      </c>
+      <c r="L4" s="32"/>
+      <c r="M4" s="8"/>
+      <c r="N4" s="9"/>
+      <c r="O4" s="25"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" s="42" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="35" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="11">
+        <v>6</v>
+      </c>
+      <c r="D5" s="11">
+        <v>8</v>
+      </c>
+      <c r="E5" s="11">
+        <v>8</v>
+      </c>
+      <c r="F5" s="11">
+        <v>6</v>
+      </c>
+      <c r="G5" s="11">
+        <v>7</v>
+      </c>
+      <c r="H5" s="11">
+        <v>5</v>
+      </c>
+      <c r="I5" s="11">
+        <v>5</v>
+      </c>
+      <c r="J5" s="11">
+        <v>7</v>
+      </c>
+      <c r="K5" s="11">
+        <v>8</v>
+      </c>
+      <c r="L5" s="12"/>
+      <c r="M5" s="13"/>
+      <c r="N5" s="14"/>
+      <c r="O5" s="25"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" s="43"/>
+      <c r="B6" s="36" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="15">
+        <v>2</v>
+      </c>
+      <c r="D6" s="15">
+        <v>2</v>
+      </c>
+      <c r="E6" s="15">
+        <v>2</v>
+      </c>
+      <c r="F6" s="15">
         <v>3</v>
       </c>
-      <c r="F4" s="17">
-        <v>9</v>
-      </c>
-      <c r="G4" s="17">
-        <v>5</v>
-      </c>
-      <c r="H4" s="17">
-        <v>7</v>
-      </c>
-      <c r="I4" s="17">
-        <v>8</v>
-      </c>
-      <c r="J4" s="17">
-        <v>6</v>
-      </c>
-      <c r="K4" s="17">
-        <v>2</v>
-      </c>
-      <c r="L4" s="18"/>
-      <c r="M4" s="14"/>
-      <c r="N4" s="15"/>
-      <c r="O4" s="40"/>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="20" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="20">
-        <v>6</v>
-      </c>
-      <c r="D5" s="20">
-        <v>8</v>
-      </c>
-      <c r="E5" s="20">
-        <v>8</v>
-      </c>
-      <c r="F5" s="20">
-        <v>6</v>
-      </c>
-      <c r="G5" s="20">
-        <v>7</v>
-      </c>
-      <c r="H5" s="20">
-        <v>5</v>
-      </c>
-      <c r="I5" s="20">
-        <v>5</v>
-      </c>
-      <c r="J5" s="20">
-        <v>7</v>
-      </c>
-      <c r="K5" s="20">
-        <v>8</v>
-      </c>
-      <c r="L5" s="21"/>
-      <c r="M5" s="22"/>
-      <c r="N5" s="23"/>
-      <c r="O5" s="40"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="24"/>
-      <c r="B6" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="25">
-        <v>2</v>
-      </c>
-      <c r="D6" s="25">
-        <v>2</v>
-      </c>
-      <c r="E6" s="25">
-        <v>2</v>
-      </c>
-      <c r="F6" s="25">
+      <c r="G6" s="15">
+        <v>2</v>
+      </c>
+      <c r="H6" s="15">
         <v>3</v>
       </c>
-      <c r="G6" s="25">
-        <v>2</v>
-      </c>
-      <c r="H6" s="25">
+      <c r="I6" s="15">
         <v>3</v>
       </c>
-      <c r="I6" s="25">
-        <v>3</v>
-      </c>
-      <c r="J6" s="25">
-        <v>2</v>
-      </c>
-      <c r="K6" s="25">
-        <v>2</v>
-      </c>
-      <c r="L6" s="26">
+      <c r="J6" s="15">
+        <v>2</v>
+      </c>
+      <c r="K6" s="15">
+        <v>2</v>
+      </c>
+      <c r="L6" s="16">
         <f>SUM(C6:K6)</f>
         <v>21</v>
       </c>
-      <c r="M6" s="22"/>
-      <c r="N6" s="23"/>
-      <c r="O6" s="40"/>
+      <c r="M6" s="13"/>
+      <c r="N6" s="14"/>
+      <c r="O6" s="25"/>
     </row>
     <row r="7" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="27"/>
-      <c r="B7" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" s="29">
+      <c r="A7" s="44"/>
+      <c r="B7" s="37" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="18">
         <f>C5-C6</f>
         <v>4</v>
       </c>
-      <c r="D7" s="28">
+      <c r="D7" s="17">
         <f t="shared" ref="D7:K7" si="0">D5-D6</f>
         <v>6</v>
       </c>
-      <c r="E7" s="28">
+      <c r="E7" s="17">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="F7" s="28">
+      <c r="F7" s="17">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="G7" s="28">
+      <c r="G7" s="17">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="H7" s="29">
+      <c r="H7" s="18">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="I7" s="29">
+      <c r="I7" s="18">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="J7" s="28">
+      <c r="J7" s="17">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="K7" s="29">
+      <c r="K7" s="18">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="L7" s="30"/>
-      <c r="M7" s="22">
-        <v>2</v>
-      </c>
-      <c r="N7" s="23">
+      <c r="L7" s="19"/>
+      <c r="M7" s="13">
+        <v>2</v>
+      </c>
+      <c r="N7" s="14">
         <v>4.4400000000000004</v>
       </c>
-      <c r="O7" s="40">
+      <c r="O7" s="25">
         <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="35" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="11">
+        <v>7</v>
+      </c>
+      <c r="D8" s="11">
         <v>8</v>
       </c>
-      <c r="C8" s="20">
+      <c r="E8" s="11">
         <v>7</v>
       </c>
-      <c r="D8" s="20">
+      <c r="F8" s="11">
+        <v>4</v>
+      </c>
+      <c r="G8" s="11">
+        <v>6</v>
+      </c>
+      <c r="H8" s="11">
+        <v>7</v>
+      </c>
+      <c r="I8" s="11">
+        <v>5</v>
+      </c>
+      <c r="J8" s="11">
+        <v>4</v>
+      </c>
+      <c r="K8" s="11">
         <v>8</v>
       </c>
-      <c r="E8" s="20">
-        <v>7</v>
-      </c>
-      <c r="F8" s="20">
-        <v>4</v>
-      </c>
-      <c r="G8" s="20">
-        <v>6</v>
-      </c>
-      <c r="H8" s="20">
-        <v>7</v>
-      </c>
-      <c r="I8" s="20">
-        <v>5</v>
-      </c>
-      <c r="J8" s="20">
-        <v>4</v>
-      </c>
-      <c r="K8" s="20">
+      <c r="L8" s="12"/>
+      <c r="M8" s="13"/>
+      <c r="N8" s="14"/>
+      <c r="O8" s="25"/>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" s="43"/>
+      <c r="B9" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="L8" s="21"/>
-      <c r="M8" s="22"/>
-      <c r="N8" s="23"/>
-      <c r="O8" s="40"/>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="24"/>
-      <c r="B9" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" s="25">
-        <v>2</v>
-      </c>
-      <c r="D9" s="25">
-        <v>2</v>
-      </c>
-      <c r="E9" s="25">
-        <v>2</v>
-      </c>
-      <c r="F9" s="25">
+      <c r="C9" s="15">
+        <v>2</v>
+      </c>
+      <c r="D9" s="15">
+        <v>2</v>
+      </c>
+      <c r="E9" s="15">
+        <v>2</v>
+      </c>
+      <c r="F9" s="15">
         <v>1</v>
       </c>
-      <c r="G9" s="25">
-        <v>2</v>
-      </c>
-      <c r="H9" s="25">
-        <v>2</v>
-      </c>
-      <c r="I9" s="25">
-        <v>2</v>
-      </c>
-      <c r="J9" s="25">
-        <v>2</v>
-      </c>
-      <c r="K9" s="25">
-        <v>2</v>
-      </c>
-      <c r="L9" s="26">
+      <c r="G9" s="15">
+        <v>2</v>
+      </c>
+      <c r="H9" s="15">
+        <v>2</v>
+      </c>
+      <c r="I9" s="15">
+        <v>2</v>
+      </c>
+      <c r="J9" s="15">
+        <v>2</v>
+      </c>
+      <c r="K9" s="15">
+        <v>2</v>
+      </c>
+      <c r="L9" s="16">
         <f>SUM(C9:K9)</f>
         <v>17</v>
       </c>
-      <c r="M9" s="22"/>
-      <c r="N9" s="23"/>
-      <c r="O9" s="40"/>
+      <c r="M9" s="13"/>
+      <c r="N9" s="14"/>
+      <c r="O9" s="25"/>
     </row>
     <row r="10" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="27"/>
-      <c r="B10" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="C10" s="28">
+      <c r="A10" s="44"/>
+      <c r="B10" s="37" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="17">
         <f>C8-C9</f>
         <v>5</v>
       </c>
-      <c r="D10" s="28">
+      <c r="D10" s="17">
         <f t="shared" ref="D10:K10" si="1">D8-D9</f>
         <v>6</v>
       </c>
-      <c r="E10" s="28">
+      <c r="E10" s="17">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="F10" s="28">
+      <c r="F10" s="17">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="G10" s="29">
+      <c r="G10" s="18">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="H10" s="28">
+      <c r="H10" s="17">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="I10" s="28">
+      <c r="I10" s="17">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="J10" s="29">
+      <c r="J10" s="18">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="K10" s="29">
+      <c r="K10" s="18">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="L10" s="30"/>
-      <c r="M10" s="22">
+      <c r="L10" s="19"/>
+      <c r="M10" s="13">
         <v>3</v>
       </c>
-      <c r="N10" s="23">
+      <c r="N10" s="14">
         <v>6.66</v>
       </c>
-      <c r="O10" s="40">
+      <c r="O10" s="25">
         <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" s="20" t="s">
+      <c r="A11" s="42" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="35" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" s="11">
         <v>8</v>
       </c>
-      <c r="C11" s="20">
+      <c r="D11" s="11">
+        <v>6</v>
+      </c>
+      <c r="E11" s="11">
+        <v>6</v>
+      </c>
+      <c r="F11" s="11">
+        <v>4</v>
+      </c>
+      <c r="G11" s="11">
+        <v>6</v>
+      </c>
+      <c r="H11" s="11">
+        <v>6</v>
+      </c>
+      <c r="I11" s="11">
+        <v>4</v>
+      </c>
+      <c r="J11" s="11">
+        <v>6</v>
+      </c>
+      <c r="K11" s="11">
         <v>8</v>
       </c>
-      <c r="D11" s="20">
-        <v>6</v>
-      </c>
-      <c r="E11" s="20">
-        <v>6</v>
-      </c>
-      <c r="F11" s="20">
-        <v>4</v>
-      </c>
-      <c r="G11" s="20">
-        <v>6</v>
-      </c>
-      <c r="H11" s="20">
-        <v>6</v>
-      </c>
-      <c r="I11" s="20">
-        <v>4</v>
-      </c>
-      <c r="J11" s="20">
-        <v>6</v>
-      </c>
-      <c r="K11" s="20">
+      <c r="L11" s="12"/>
+      <c r="M11" s="13"/>
+      <c r="N11" s="14"/>
+      <c r="O11" s="25"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" s="43"/>
+      <c r="B12" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="L11" s="21"/>
-      <c r="M11" s="22"/>
-      <c r="N11" s="23"/>
-      <c r="O11" s="40"/>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="24"/>
-      <c r="B12" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="C12" s="25">
-        <v>2</v>
-      </c>
-      <c r="D12" s="25">
+      <c r="C12" s="15">
+        <v>2</v>
+      </c>
+      <c r="D12" s="15">
         <v>1</v>
       </c>
-      <c r="E12" s="25">
+      <c r="E12" s="15">
         <v>1</v>
       </c>
-      <c r="F12" s="25">
-        <v>2</v>
-      </c>
-      <c r="G12" s="25">
-        <v>2</v>
-      </c>
-      <c r="H12" s="25">
-        <v>2</v>
-      </c>
-      <c r="I12" s="25">
-        <v>2</v>
-      </c>
-      <c r="J12" s="25">
-        <v>2</v>
-      </c>
-      <c r="K12" s="25">
+      <c r="F12" s="15">
+        <v>2</v>
+      </c>
+      <c r="G12" s="15">
+        <v>2</v>
+      </c>
+      <c r="H12" s="15">
+        <v>2</v>
+      </c>
+      <c r="I12" s="15">
+        <v>2</v>
+      </c>
+      <c r="J12" s="15">
+        <v>2</v>
+      </c>
+      <c r="K12" s="15">
         <v>1</v>
       </c>
-      <c r="L12" s="26">
+      <c r="L12" s="16">
         <f>SUM(C12:K12)</f>
         <v>15</v>
       </c>
-      <c r="M12" s="22"/>
-      <c r="N12" s="23"/>
-      <c r="O12" s="40"/>
+      <c r="M12" s="13"/>
+      <c r="N12" s="14"/>
+      <c r="O12" s="25"/>
     </row>
     <row r="13" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="27"/>
-      <c r="B13" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="C13" s="28">
+      <c r="A13" s="44"/>
+      <c r="B13" s="37" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="17">
         <f>C11-C12</f>
         <v>6</v>
       </c>
-      <c r="D13" s="29">
+      <c r="D13" s="18">
         <f t="shared" ref="D13:K13" si="2">D11-D12</f>
         <v>5</v>
       </c>
-      <c r="E13" s="28">
+      <c r="E13" s="17">
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
-      <c r="F13" s="29">
+      <c r="F13" s="18">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
-      <c r="G13" s="29">
+      <c r="G13" s="18">
         <f t="shared" si="2"/>
         <v>4</v>
       </c>
-      <c r="H13" s="28">
+      <c r="H13" s="17">
         <f t="shared" si="2"/>
         <v>4</v>
       </c>
-      <c r="I13" s="29">
+      <c r="I13" s="18">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
-      <c r="J13" s="28">
+      <c r="J13" s="17">
         <f t="shared" si="2"/>
         <v>4</v>
       </c>
-      <c r="K13" s="28">
+      <c r="K13" s="17">
         <f t="shared" si="2"/>
         <v>7</v>
       </c>
-      <c r="L13" s="30"/>
-      <c r="M13" s="22">
-        <v>2</v>
-      </c>
-      <c r="N13" s="23">
+      <c r="L13" s="19"/>
+      <c r="M13" s="13">
+        <v>2</v>
+      </c>
+      <c r="N13" s="14">
         <v>4.4400000000000004</v>
       </c>
-      <c r="O13" s="40">
+      <c r="O13" s="25">
         <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="19" t="s">
-        <v>23</v>
-      </c>
-      <c r="B14" s="20" t="s">
+      <c r="A14" s="42" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="35" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="11">
+        <v>5</v>
+      </c>
+      <c r="D14" s="11">
+        <v>7</v>
+      </c>
+      <c r="E14" s="11">
+        <v>5</v>
+      </c>
+      <c r="F14" s="11">
+        <v>4</v>
+      </c>
+      <c r="G14" s="11">
+        <v>7</v>
+      </c>
+      <c r="H14" s="11">
+        <v>6</v>
+      </c>
+      <c r="I14" s="11">
+        <v>4</v>
+      </c>
+      <c r="J14" s="11">
+        <v>5</v>
+      </c>
+      <c r="K14" s="11">
         <v>8</v>
       </c>
-      <c r="C14" s="20">
-        <v>5</v>
-      </c>
-      <c r="D14" s="20">
-        <v>7</v>
-      </c>
-      <c r="E14" s="20">
-        <v>5</v>
-      </c>
-      <c r="F14" s="20">
-        <v>4</v>
-      </c>
-      <c r="G14" s="20">
-        <v>7</v>
-      </c>
-      <c r="H14" s="20">
-        <v>6</v>
-      </c>
-      <c r="I14" s="20">
-        <v>4</v>
-      </c>
-      <c r="J14" s="20">
-        <v>5</v>
-      </c>
-      <c r="K14" s="20">
+      <c r="L14" s="12"/>
+      <c r="M14" s="13"/>
+      <c r="N14" s="14"/>
+      <c r="O14" s="25"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" s="43"/>
+      <c r="B15" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="L14" s="21"/>
-      <c r="M14" s="22"/>
-      <c r="N14" s="23"/>
-      <c r="O14" s="40"/>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="24"/>
-      <c r="B15" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="C15" s="25">
+      <c r="C15" s="15">
         <v>1</v>
       </c>
-      <c r="D15" s="25">
+      <c r="D15" s="15">
         <v>1</v>
       </c>
-      <c r="E15" s="25">
+      <c r="E15" s="15">
         <v>1</v>
       </c>
-      <c r="F15" s="25">
-        <v>2</v>
-      </c>
-      <c r="G15" s="25">
+      <c r="F15" s="15">
+        <v>2</v>
+      </c>
+      <c r="G15" s="15">
         <v>1</v>
       </c>
-      <c r="H15" s="25">
-        <v>2</v>
-      </c>
-      <c r="I15" s="25">
-        <v>2</v>
-      </c>
-      <c r="J15" s="25">
-        <v>2</v>
-      </c>
-      <c r="K15" s="25">
+      <c r="H15" s="15">
+        <v>2</v>
+      </c>
+      <c r="I15" s="15">
+        <v>2</v>
+      </c>
+      <c r="J15" s="15">
+        <v>2</v>
+      </c>
+      <c r="K15" s="15">
         <v>1</v>
       </c>
-      <c r="L15" s="26">
+      <c r="L15" s="16">
         <f>SUM(C15:K15)</f>
         <v>13</v>
       </c>
-      <c r="M15" s="22"/>
-      <c r="N15" s="23"/>
-      <c r="O15" s="40"/>
+      <c r="M15" s="13"/>
+      <c r="N15" s="14"/>
+      <c r="O15" s="25"/>
     </row>
     <row r="16" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="27"/>
-      <c r="B16" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="C16" s="29">
+      <c r="A16" s="44"/>
+      <c r="B16" s="37" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" s="18">
         <f>C14-C15</f>
         <v>4</v>
       </c>
-      <c r="D16" s="28">
+      <c r="D16" s="17">
         <f t="shared" ref="D16:K16" si="3">D14-D15</f>
         <v>6</v>
       </c>
-      <c r="E16" s="29">
+      <c r="E16" s="18">
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
-      <c r="F16" s="29">
+      <c r="F16" s="18">
         <f t="shared" si="3"/>
         <v>2</v>
       </c>
-      <c r="G16" s="28">
+      <c r="G16" s="17">
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="H16" s="28">
+      <c r="H16" s="17">
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
-      <c r="I16" s="29">
+      <c r="I16" s="18">
         <f t="shared" si="3"/>
         <v>2</v>
       </c>
-      <c r="J16" s="28">
+      <c r="J16" s="17">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="K16" s="28">
+      <c r="K16" s="17">
         <f t="shared" si="3"/>
         <v>7</v>
       </c>
-      <c r="L16" s="30"/>
-      <c r="M16" s="31">
-        <v>2</v>
-      </c>
-      <c r="N16" s="32">
+      <c r="L16" s="19"/>
+      <c r="M16" s="20">
+        <v>2</v>
+      </c>
+      <c r="N16" s="21">
         <v>4.4400000000000004</v>
       </c>
-      <c r="O16" s="41">
+      <c r="O16" s="26">
         <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="33"/>
-      <c r="B17" s="33"/>
-      <c r="C17" s="33"/>
-      <c r="D17" s="33"/>
-      <c r="E17" s="33"/>
-      <c r="F17" s="33"/>
-      <c r="G17" s="33"/>
-      <c r="H17" s="33"/>
-      <c r="I17" s="33"/>
-      <c r="J17" s="33"/>
-      <c r="K17" s="33"/>
-      <c r="L17" s="33"/>
-      <c r="M17" s="34"/>
-      <c r="N17" s="35"/>
-      <c r="O17" s="42"/>
+      <c r="A17" s="45"/>
+      <c r="B17" s="45"/>
+      <c r="C17" s="45"/>
+      <c r="D17" s="45"/>
+      <c r="E17" s="45"/>
+      <c r="F17" s="45"/>
+      <c r="G17" s="45"/>
+      <c r="H17" s="45"/>
+      <c r="I17" s="45"/>
+      <c r="J17" s="45"/>
+      <c r="K17" s="45"/>
+      <c r="L17" s="45"/>
+      <c r="M17" s="22"/>
+      <c r="N17" s="23"/>
+      <c r="O17" s="27"/>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="33"/>
-      <c r="B18" s="33"/>
-      <c r="C18" s="36" t="s">
+      <c r="A18" s="45"/>
+      <c r="B18" s="45"/>
+      <c r="C18" s="46" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" s="46" t="s">
         <v>11</v>
       </c>
-      <c r="D18" s="33" t="s">
+      <c r="E18" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="E18" s="33" t="s">
+      <c r="F18" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="F18" s="33" t="s">
+      <c r="G18" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="G18" s="33" t="s">
+      <c r="H18" s="46" t="s">
         <v>15</v>
       </c>
-      <c r="H18" s="33" t="s">
+      <c r="I18" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="I18" s="33" t="s">
+      <c r="J18" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="J18" s="33" t="s">
+      <c r="K18" s="46" t="s">
         <v>18</v>
       </c>
-      <c r="K18" s="33" t="s">
-        <v>19</v>
-      </c>
-      <c r="L18" s="33"/>
-      <c r="M18" s="34"/>
-      <c r="N18" s="35"/>
-      <c r="O18" s="42"/>
+      <c r="L18" s="45"/>
+      <c r="M18" s="22"/>
+      <c r="N18" s="33"/>
+      <c r="O18" s="34"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="33"/>
-      <c r="B19" s="33"/>
-      <c r="C19" s="37" t="s">
-        <v>19</v>
-      </c>
-      <c r="D19" s="38"/>
-      <c r="E19" s="38"/>
-      <c r="F19" s="33" t="s">
-        <v>11</v>
-      </c>
-      <c r="G19" s="33" t="s">
+      <c r="A19" s="45"/>
+      <c r="B19" s="45"/>
+      <c r="C19" s="47" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" s="47"/>
+      <c r="E19" s="47"/>
+      <c r="F19" s="46" t="s">
+        <v>10</v>
+      </c>
+      <c r="G19" s="46" t="s">
+        <v>13</v>
+      </c>
+      <c r="H19" s="46"/>
+      <c r="I19" s="46"/>
+      <c r="J19" s="46"/>
+      <c r="K19" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="H19" s="33"/>
-      <c r="I19" s="33"/>
-      <c r="J19" s="33"/>
-      <c r="K19" s="33" t="s">
-        <v>15</v>
-      </c>
-      <c r="L19" s="33"/>
-      <c r="M19" s="34"/>
-      <c r="N19" s="35">
+      <c r="L19" s="45"/>
+      <c r="M19" s="22"/>
+      <c r="N19" s="33">
         <f>SUM(N7:N18)</f>
         <v>19.980000000000004</v>
       </c>
-      <c r="O19" s="42">
+      <c r="O19" s="34">
         <f>SUM(O7:O18)</f>
         <v>19</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
+    <mergeCell ref="L2:L4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>